<commit_message>
Dates des écritures : date de l'opération réelle (VC-12, VC-16, décision du 26/10)
- VC-12 : la modification d'une vente d'un autre jour date la recette et les mouvements de stock (vente de la copie,
  retour de l'annulation) de la vente d'origine, comme la transaction et la contre-passation. Une modification du
  jour même ne change pas.
- VC-16 : la transaction d'un mouvement de caisse porte la date saisie du mouvement (le futur reste refusé).
- repro-vente-comptant : VC-12 compare toutes les dates des écritures, stock de l'annulation compris.
- Cahier de recette mis à jour (vierge et rempli : 59 OK, 2 bloqués par le poste, 1 non joué) et document §9.6.
</commit_message>
<xml_diff>
--- a/docs/notices/CAHIER_RECETTE_AUDITS_2026-10-26.xlsx
+++ b/docs/notices/CAHIER_RECETTE_AUDITS_2026-10-26.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1050" uniqueCount="578">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1050" uniqueCount="577">
   <si>
     <t>Cahier de recette : corrections des audits de code</t>
   </si>
@@ -28,7 +28,7 @@
     <t>Version testée</t>
   </si>
   <si>
-    <t>Branche PRES-/audits-code-dffa0a, commit 9b02b3c7 (26/10/2026). WAR : target/prestige.war construit à partir de ce commit. Il ne contient pas les commits récents de la branche principale (droits, horloge, bornes, téléphone de la vente).</t>
+    <t>Branche PRES-/audits-code-dffa0a, état du 26/10/2026 au soir (dates VC-12 et VC-16 comprises). WAR : target/prestige.war construit à partir de cet état. Il ne contient pas les commits récents de la branche principale (droits, horloge, bornes, téléphone de la vente).</t>
   </si>
   <si>
     <t>Référence</t>
@@ -79,10 +79,10 @@
     <t>Colonne « Test automatique » : script Playwright du dépôt (src/test/e2e/...), lancé seul, un à la fois : node src/test/e2e/audits/repro-vente-comptant.js. Une ligne FAIL = défaut présent.</t>
   </si>
   <si>
-    <t>Restent en échec</t>
-  </si>
-  <si>
-    <t>VC-12 et VC-16 (cas « hier ») : décision métier en attente sur la date des écritures. Voir l'onglet « Décisions ».</t>
+    <t>Dates des écritures</t>
+  </si>
+  <si>
+    <t>VC-12 et VC-16 : décision du 26/10, les écritures portent la date de l'opération réelle (vente d'origine, date saisie du mouvement).</t>
   </si>
   <si>
     <t>Exemple de saisie</t>
@@ -411,13 +411,13 @@
 3. Comparer les dates de la transaction, de la contre-passation, de la recette et du mouvement de stock.</t>
   </si>
   <si>
-    <t>DÉCISION EN ATTENTE (date de l'opération ou de la saisie) : non corrigé. À jouer pour constat seulement.</t>
+    <t>Toutes les écritures portent la date de la vente d'origine (veille) : transaction de la copie, contre-passation, recette, mouvements de stock de la copie et de l'annulation (décision du 26/10 : date de l'opération réelle). Une modification du jour même reste datée du jour.</t>
   </si>
   <si>
     <t>Transaction et contre-passation datées de la veille ; recette et stock du jour.</t>
   </si>
   <si>
-    <t>repro-vente-comptant.js (VC-12) : reste en échec tant que la décision n'est pas prise</t>
+    <t>repro-vente-comptant.js (VC-12)</t>
   </si>
   <si>
     <t>11</t>
@@ -463,13 +463,13 @@
 2. Puis une entrée de 1 000 F datée d'hier.</t>
   </si>
   <si>
-    <t>Date de demain refusée. Date d'hier : DÉCISION EN ATTENTE (aujourd'hui, mouvement et règlement à hier, transaction au jour).</t>
+    <t>Date de demain refusée avec un message. Date d'hier : mouvement, règlement et transaction de caisse datés d'hier (décision du 26/10 : date saisie du mouvement).</t>
   </si>
   <si>
     <t>Date future acceptée ; dates différentes entre mouvement, règlement et transaction.</t>
   </si>
   <si>
-    <t>repro-remise-caisse.js (VC-16) : le cas « hier » reste en échec tant que la décision n'est pas prise</t>
+    <t>repro-remise-caisse.js (VC-16)</t>
   </si>
   <si>
     <t>13</t>
@@ -1743,10 +1743,7 @@
     <t>VC-12, VC-16</t>
   </si>
   <si>
-    <t>Seules les dates futures sont refusées. Une modification d'une vente de la veille et un mouvement daté d'hier gardent des dates différentes selon l'écriture.</t>
-  </si>
-  <si>
-    <t>Date de l'opération réelle, ou date de la saisie ?</t>
+    <t>Tranché le 26/10 : date de l'opération réelle. Modification d'une vente d'un autre jour : toutes les écritures à la date de la vente d'origine ; mouvement de caisse : date saisie (le futur est refusé).</t>
   </si>
   <si>
     <t>Vente différée réglée puis modifiée</t>
@@ -5478,7 +5475,7 @@
         <v>558</v>
       </c>
       <c r="D2" t="s" s="5">
-        <v>559</v>
+        <v>497</v>
       </c>
       <c r="E2" t="s" s="6">
         <v>52</v>
@@ -5492,16 +5489,16 @@
     </row>
     <row r="3">
       <c r="A3" t="s" s="5">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B3" t="s" s="5">
         <v>424</v>
       </c>
       <c r="C3" t="s" s="5">
+        <v>560</v>
+      </c>
+      <c r="D3" t="s" s="5">
         <v>561</v>
-      </c>
-      <c r="D3" t="s" s="5">
-        <v>562</v>
       </c>
       <c r="E3" t="s" s="6">
         <v>52</v>
@@ -5515,16 +5512,16 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="5">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B4" t="s" s="5">
         <v>432</v>
       </c>
       <c r="C4" t="s" s="5">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="D4" t="s" s="5">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="E4" t="s" s="6">
         <v>52</v>
@@ -5538,16 +5535,16 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="5">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B5" t="s" s="5">
         <v>358</v>
       </c>
       <c r="C5" t="s" s="5">
+        <v>565</v>
+      </c>
+      <c r="D5" t="s" s="5">
         <v>566</v>
-      </c>
-      <c r="D5" t="s" s="5">
-        <v>567</v>
       </c>
       <c r="E5" t="s" s="6">
         <v>52</v>
@@ -5561,13 +5558,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="5">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B6" t="s" s="5">
         <v>202</v>
       </c>
       <c r="C6" t="s" s="5">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="D6" t="s" s="5">
         <v>497</v>
@@ -5584,16 +5581,16 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="5">
+        <v>569</v>
+      </c>
+      <c r="B7" t="s" s="5">
         <v>570</v>
       </c>
-      <c r="B7" t="s" s="5">
+      <c r="C7" t="s" s="5">
         <v>571</v>
       </c>
-      <c r="C7" t="s" s="5">
+      <c r="D7" t="s" s="5">
         <v>572</v>
-      </c>
-      <c r="D7" t="s" s="5">
-        <v>573</v>
       </c>
       <c r="E7" t="s" s="6">
         <v>52</v>
@@ -5607,16 +5604,16 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="5">
+        <v>573</v>
+      </c>
+      <c r="B8" t="s" s="5">
         <v>574</v>
       </c>
-      <c r="B8" t="s" s="5">
+      <c r="C8" t="s" s="5">
         <v>575</v>
       </c>
-      <c r="C8" t="s" s="5">
+      <c r="D8" t="s" s="5">
         <v>576</v>
-      </c>
-      <c r="D8" t="s" s="5">
-        <v>577</v>
       </c>
       <c r="E8" t="s" s="6">
         <v>52</v>

</xml_diff>